<commit_message>
Shopee files: hold back every product that uses piece 02
The owner says piece 02 (กังหัน) is not usable yet. Ready drops 24 and 29 (11 left),
prototype drops 5, 6, 7 and 25 (13 left); the summary page lists the six held products.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFe2Neq3JpzqWomS7eNDYn
</commit_message>
<xml_diff>
--- a/shopee-20261021/oct26-shopee-prototype.xlsx
+++ b/shopee-20261021/oct26-shopee-prototype.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4405" uniqueCount="4405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4369" uniqueCount="4369">
   <si>
     <t>ภาพรวม</t>
   </si>
@@ -12857,120 +12857,6 @@
     <t xml:space="preserve">เปิด</t>
   </si>
   <si>
-    <t xml:space="preserve">ซองอั่งเปาพับกังหัน หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">อั่งเปาที่ผู้รับเก็บไว้ใช้ต่อ ไม่ทิ้ง
-• คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: กังหัน 02 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: 5.4 × 5.4 ซม. เมื่อพับ
-• เหมาะกับ: ของขวัญองค์กร ตรุษจีน
-วิธีประกอบ
-1. พับธนบัตรให้เล็กกว่า 5 ซม.
-2. วางกลางแผ่น พับกลีบเข้ากลางทีละกลีบ
-3. กลีบสุดท้ายสอดใต้กลีบแรก
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">69</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/05.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ซองใส่เครื่องประดับ หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ห่อแหวนด้วยหนังแท้แทนกล่องกระดาษ
-• คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: กังหัน 02 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: 5.4 × 5.4 ซม.
-• เหมาะกับ: ร้านเครื่องประดับ งานแต่ง
-วิธีประกอบ
-1. วางแหวนหรือต่างหูตรงกลาง
-2. พับกลีบเข้ากลางแบบกังหัน
-3. กลีบสุดท้ายสอดล็อก
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">69</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/06.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ซองการ์ดติดของขวัญ หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">การ์ดอวยพรที่ห่อมาอย่างตั้งใจ
-• คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: กังหัน 02 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: 5.4 × 5.4 ซม.
-• เหมาะกับ: ร้านดอกไม้ ร้านของขวัญ
-วิธีประกอบ
-1. เขียนการ์ด 5 × 5 ซม.
-2. วางการ์ดแล้วพับกลีบแบบกังหัน
-3. ผูกเชือกติดกล่องหรือช่อดอกไม้
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">59</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/07.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
     <t xml:space="preserve">กล่องแหวนหนังแท้ หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
   </si>
   <si>
@@ -13422,44 +13308,6 @@
   </si>
   <si>
     <t xml:space="preserve">0.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">กังหันลมหนัง หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ของเล่นที่ลูกเป่าเล่นได้ทั้งวัน
-• คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: กังหัน 02 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: 9 ซม.
-• เหมาะกับ: เด็ก ของฝาก
-วิธีประกอบ
-1. พับปลายกลีบเข้าหาจุดกลางทีละกลีบ
-2. ตอกหมุดผ่านจุดกลาง
-3. เป่าดูให้หมุน
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/25.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
   </si>
   <si>
     <t xml:space="preserve">เปิด</t>
@@ -14537,7 +14385,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK23"/>
+  <dimension ref="A1:AK19"/>
   <cols>
     <col customWidth="true" max="37" min="37" style="8" width="20"/>
     <col customWidth="true" max="36" min="36" style="5" width="20"/>
@@ -16199,122 +16047,6 @@
         <v>4368</v>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="6" t="s">
-        <v>4369</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>4370</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>4371</v>
-      </c>
-      <c r="P20" s="6" t="s">
-        <v>4372</v>
-      </c>
-      <c r="Q20" s="5" t="s">
-        <v>4373</v>
-      </c>
-      <c r="R20" s="6" t="s">
-        <v>4374</v>
-      </c>
-      <c r="V20" s="6" t="s">
-        <v>4375</v>
-      </c>
-      <c r="AE20" s="6" t="s">
-        <v>4376</v>
-      </c>
-      <c r="AI20" s="6" t="s">
-        <v>4377</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="6" t="s">
-        <v>4378</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>4379</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>4380</v>
-      </c>
-      <c r="P21" s="6" t="s">
-        <v>4381</v>
-      </c>
-      <c r="Q21" s="5" t="s">
-        <v>4382</v>
-      </c>
-      <c r="R21" s="6" t="s">
-        <v>4383</v>
-      </c>
-      <c r="V21" s="6" t="s">
-        <v>4384</v>
-      </c>
-      <c r="AE21" s="6" t="s">
-        <v>4385</v>
-      </c>
-      <c r="AI21" s="6" t="s">
-        <v>4386</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="6" t="s">
-        <v>4387</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>4388</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>4389</v>
-      </c>
-      <c r="P22" s="6" t="s">
-        <v>4390</v>
-      </c>
-      <c r="Q22" s="5" t="s">
-        <v>4391</v>
-      </c>
-      <c r="R22" s="6" t="s">
-        <v>4392</v>
-      </c>
-      <c r="V22" s="6" t="s">
-        <v>4393</v>
-      </c>
-      <c r="AE22" s="6" t="s">
-        <v>4394</v>
-      </c>
-      <c r="AI22" s="6" t="s">
-        <v>4395</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="6" t="s">
-        <v>4396</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>4397</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>4398</v>
-      </c>
-      <c r="P23" s="6" t="s">
-        <v>4399</v>
-      </c>
-      <c r="Q23" s="5" t="s">
-        <v>4400</v>
-      </c>
-      <c r="R23" s="6" t="s">
-        <v>4401</v>
-      </c>
-      <c r="V23" s="6" t="s">
-        <v>4402</v>
-      </c>
-      <c r="AE23" s="6" t="s">
-        <v>4403</v>
-      </c>
-      <c r="AI23" s="6" t="s">
-        <v>4404</v>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection sheet="true" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
   <dataValidations count="2">

</xml_diff>